<commit_message>
refactor: extract legacy army lists from v2024
</commit_message>
<xml_diff>
--- a/data/raw/army-lists.xlsx
+++ b/data/raw/army-lists.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Army Lists" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="81">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -41,6 +41,9 @@
     <t xml:space="preserve">page</t>
   </si>
   <si>
+    <t xml:space="preserve">warband_mode</t>
+  </si>
+  <si>
     <t xml:space="preserve">bow_limit</t>
   </si>
   <si>
@@ -50,6 +53,48 @@
     <t xml:space="preserve">break_point</t>
   </si>
   <si>
+    <t xml:space="preserve">single_warband_profiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">single_warband_races</t>
+  </si>
+  <si>
+    <t xml:space="preserve">single_warband_factions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">single_warband_unit_types</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the-fellowship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">good</t>
+  </si>
+  <si>
+    <t xml:space="preserve">armies-of-the-lord-of-the-rings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">single</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the-shire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">choice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">road-to-rivendell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">breaking-of-the-fellowship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">standard</t>
+  </si>
+  <si>
     <t xml:space="preserve">army_list</t>
   </si>
   <si>
@@ -59,6 +104,9 @@
     <t xml:space="preserve">tier</t>
   </si>
   <si>
+    <t xml:space="preserve">capabilities</t>
+  </si>
+  <si>
     <t xml:space="preserve">add_keywords</t>
   </si>
   <si>
@@ -68,6 +116,51 @@
     <t xml:space="preserve">remove_wargear</t>
   </si>
   <si>
+    <t xml:space="preserve">gandalf-the-grey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hero-of-legend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leader; follower</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aragorn-strider</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hero-of-valour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">legolas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gimli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">boromir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">frodo-baggins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hero-of-fortitude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">samwise-gamgee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">meriadoc-brandybuck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">independent-hero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peregrin-took</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bill-the-pony</t>
+  </si>
+  <si>
     <t xml:space="preserve">option</t>
   </si>
   <si>
@@ -83,6 +176,24 @@
     <t xml:space="preserve">upgrade_from</t>
   </si>
   <si>
+    <t xml:space="preserve">bow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mithril-coat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sting</t>
+  </si>
+  <si>
     <t xml:space="preserve">leader</t>
   </si>
   <si>
@@ -141,6 +252,24 @@
   </si>
   <si>
     <t xml:space="preserve">category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">single-warband</t>
+  </si>
+  <si>
+    <t xml:space="preserve">additional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">you-have-my-sword</t>
+  </si>
+  <si>
+    <t xml:space="preserve">special</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bond-of-fellowship</t>
+  </si>
+  <si>
+    <t xml:space="preserve">traverse-the-wilderness</t>
   </si>
 </sst>
 </file>
@@ -150,7 +279,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -172,6 +301,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -216,7 +351,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -226,6 +361,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -246,16 +389,22 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15.23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.68"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="8.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.61"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="1" width="8.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.44"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="8.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.65"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="20.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="22.62"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="13" style="1" width="8.5"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -274,11 +423,97 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>82</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>84</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>86</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>88</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -297,35 +532,221 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="8.3671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="1" style="1" width="8.36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="1" width="19.06"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="1" width="8.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="18.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="1" width="19.06"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="9" style="1" width="8.36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>12</v>
+        <v>27</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="4"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -344,38 +765,133 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A36:H36"/>
-  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H36"/>
+  <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="0" width="15.43"/>
   </cols>
   <sheetData>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="C36" s="0" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="D36" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="F36" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="G36" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="H36" s="0" t="s">
-        <v>17</v>
-      </c>
-    </row>
+      <c r="D1" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -393,29 +909,29 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="1" style="1" width="12.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -435,35 +951,35 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="1" style="0" width="17.75"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>25</v>
+        <v>62</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -483,44 +999,44 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultColWidth="15.94921875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.95703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B1" s="0" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>27</v>
+        <v>64</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>32</v>
+        <v>69</v>
       </c>
       <c r="K1" s="0" t="s">
-        <v>33</v>
+        <v>70</v>
       </c>
       <c r="L1" s="0" t="s">
-        <v>34</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -540,23 +1056,23 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B1" s="0" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -575,22 +1091,68 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.3671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.8"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="2" style="1" width="8.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20.87"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="4" style="1" width="8.36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>37</v>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>